<commit_message>
Updated PTax automation code
</commit_message>
<xml_diff>
--- a/src/test/resources/WI Data.xlsx
+++ b/src/test/resources/WI Data.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="110" windowWidth="14810" windowHeight="8010"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="15200" windowHeight="5360"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -72,7 +73,7 @@
     <t>001</t>
   </si>
   <si>
-    <t>0002</t>
+    <t>0001</t>
   </si>
 </sst>
 </file>

</xml_diff>